<commit_message>
updating template formats and fixing compatibility for reports generation
</commit_message>
<xml_diff>
--- a/templates_formats/Info_estudiante.xlsx
+++ b/templates_formats/Info_estudiante.xlsx
@@ -152,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -181,29 +181,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="15"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" indent="19"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="27"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="26"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" indent="23"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" indent="18"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" indent="16"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" indent="12"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -509,10 +497,10 @@
   <dimension ref="A1:R69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.5" customWidth="1"/>
+    <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
     <col min="3" max="3" width="1.625" customWidth="1"/>
-    <col min="4" max="4" width="47.5" customWidth="1"/>
+    <col min="4" max="4" width="37.625" customWidth="1"/>
     <col min="5" max="5" width="22.625" customWidth="1"/>
     <col min="6" max="6" width="9.625" customWidth="1"/>
     <col min="7" max="7" width="9.25" customWidth="1"/>
@@ -521,56 +509,94 @@
     <col min="12" max="16" width="2.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="D1" s="16" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="D2" s="17" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
         <v>24</v>
       </c>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="D3" s="18" t="s">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="D4" s="19" t="s">
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="K5" s="1"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D6" s="12"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="9" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="D5" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="2"/>
-      <c r="H5" s="1"/>
-      <c r="K5" s="1"/>
-    </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="D6" s="14"/>
-      <c r="E6" s="2"/>
       <c r="H6" s="1"/>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="D7" s="15" t="s">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="E7" s="2"/>
-      <c r="H7" s="1"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="E8" s="4"/>
       <c r="F8" s="2"/>
       <c r="H8" s="1"/>
@@ -578,7 +604,7 @@
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>13</v>
       </c>
@@ -594,7 +620,7 @@
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
         <v>4</v>
       </c>
@@ -605,7 +631,7 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
         <v>5</v>
       </c>
@@ -618,7 +644,7 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
         <v>7</v>
       </c>
@@ -632,7 +658,7 @@
       <c r="K12" s="1"/>
       <c r="Q12" s="5"/>
     </row>
-    <row r="13" spans="2:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="7"/>
       <c r="D13" s="11" t="s">
         <v>9</v>
@@ -651,7 +677,7 @@
       <c r="P13" s="8"/>
       <c r="Q13" s="1"/>
     </row>
-    <row r="14" spans="2:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="7"/>
       <c r="D14" s="11" t="s">
         <v>11</v>
@@ -670,7 +696,7 @@
       <c r="P14" s="7"/>
       <c r="Q14" s="1"/>
     </row>
-    <row r="15" spans="2:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15" s="7"/>
       <c r="D15" s="11" t="s">
         <v>14</v>
@@ -688,7 +714,7 @@
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
     </row>
-    <row r="16" spans="2:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="7"/>
       <c r="D16" s="11"/>
       <c r="E16" s="7"/>
@@ -703,14 +729,16 @@
       <c r="P16" s="7"/>
       <c r="Q16" s="1"/>
     </row>
-    <row r="17" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="7"/>
-      <c r="D17" s="12" t="s">
+    <row r="17" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
       <c r="H17" s="7"/>
       <c r="I17" s="1"/>
       <c r="L17" s="7"/>
@@ -720,7 +748,7 @@
       <c r="P17" s="7"/>
       <c r="Q17" s="1"/>
     </row>
-    <row r="18" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
@@ -735,7 +763,7 @@
       <c r="P18" s="7"/>
       <c r="Q18" s="1"/>
     </row>
-    <row r="19" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="7"/>
       <c r="D19" s="11" t="s">
         <v>16</v>
@@ -754,7 +782,7 @@
       <c r="P19" s="7"/>
       <c r="Q19" s="1"/>
     </row>
-    <row r="20" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="7"/>
       <c r="D20" s="11" t="s">
         <v>18</v>
@@ -773,7 +801,7 @@
       <c r="P20" s="7"/>
       <c r="Q20" s="1"/>
     </row>
-    <row r="21" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="7"/>
       <c r="D21" s="11" t="s">
         <v>20</v>
@@ -792,7 +820,7 @@
       <c r="P21" s="7"/>
       <c r="Q21" s="1"/>
     </row>
-    <row r="22" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="7"/>
       <c r="D22" s="11" t="s">
         <v>22</v>
@@ -809,7 +837,7 @@
       <c r="P22" s="7"/>
       <c r="Q22" s="1"/>
     </row>
-    <row r="23" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
       <c r="E23" s="7"/>
@@ -824,7 +852,7 @@
       <c r="P23" s="7"/>
       <c r="Q23" s="1"/>
     </row>
-    <row r="24" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
       <c r="E24" s="7"/>
@@ -839,7 +867,7 @@
       <c r="P24" s="7"/>
       <c r="Q24" s="1"/>
     </row>
-    <row r="25" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
       <c r="E25" s="7"/>
@@ -854,7 +882,7 @@
       <c r="P25" s="7"/>
       <c r="Q25" s="1"/>
     </row>
-    <row r="26" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
       <c r="E26" s="7"/>
@@ -870,7 +898,7 @@
       <c r="P26" s="7"/>
       <c r="Q26" s="1"/>
     </row>
-    <row r="27" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
       <c r="E27" s="7"/>
@@ -879,7 +907,7 @@
       <c r="H27" s="7"/>
       <c r="I27" s="1"/>
     </row>
-    <row r="28" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
       <c r="E28" s="7"/>
@@ -888,7 +916,7 @@
       <c r="H28" s="7"/>
       <c r="I28" s="1"/>
     </row>
-    <row r="29" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
       <c r="E29" s="7"/>
@@ -897,7 +925,7 @@
       <c r="H29" s="7"/>
       <c r="I29" s="1"/>
     </row>
-    <row r="30" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
       <c r="E30" s="7"/>
@@ -906,7 +934,7 @@
       <c r="H30" s="7"/>
       <c r="I30" s="1"/>
     </row>
-    <row r="31" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
@@ -915,7 +943,7 @@
       <c r="H31" s="7"/>
       <c r="I31" s="1"/>
     </row>
-    <row r="32" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
       <c r="E32" s="7"/>
@@ -1164,6 +1192,15 @@
       <c r="Q69" s="1"/>
     </row>
   </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A7:H7"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="172" orientation="landscape" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
 </worksheet>

</xml_diff>